<commit_message>
Initial commit - Saucedemo manual testing project
</commit_message>
<xml_diff>
--- a/SauceDemo_TestCase_Document.xlsx
+++ b/SauceDemo_TestCase_Document.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\QA Projects\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\QA Projects\SauceDemo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217789A5-21AF-4348-A610-788FEBAB5460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5D97F6-9A76-4087-B159-F8930AA3B238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{61EE1E3B-FF1C-4575-838F-6EAC3CE006BA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{61EE1E3B-FF1C-4575-838F-6EAC3CE006BA}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Plan Summary" sheetId="4" r:id="rId1"/>
@@ -750,13 +750,17 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -768,10 +772,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1098,167 +1098,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
     </row>
     <row r="2" spans="1:5" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
     </row>
     <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
     </row>
     <row r="4" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
     </row>
     <row r="5" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
     </row>
     <row r="6" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
     </row>
     <row r="7" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
     </row>
     <row r="8" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
     </row>
     <row r="9" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
     </row>
     <row r="10" spans="1:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="A10" s="15"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
     </row>
     <row r="11" spans="1:5" ht="21" x14ac:dyDescent="0.4">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
     </row>
     <row r="12" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="B12" s="22">
+      <c r="B12" s="17">
         <v>21</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
     </row>
     <row r="13" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="22">
+      <c r="B13" s="17">
         <v>16</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
     </row>
     <row r="14" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="B14" s="22">
+      <c r="B14" s="17">
         <v>0</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
     </row>
     <row r="15" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="B15" s="22">
+      <c r="B15" s="17">
         <v>5</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="B15:E15"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -1269,6 +1264,11 @@
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="B9:E9"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B15:E15"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" xr:uid="{EFAB7DC7-25C8-4364-B651-3688DFD9D08C}"/>

</xml_diff>